<commit_message>
feat: update analyze_records script and add new summary generation functionality
</commit_message>
<xml_diff>
--- a/0_1_SELECT_ZIVE_DATA_2026/AtsisiustiDuomenys_2026/KJ_-_2026-03-13_2225_to_2026-03-14_0636_8h_10min_test/KJ_-_2026-03-13_2225_to_2026-03-14_0636_8h_10min_test_records_summary.xlsx
+++ b/0_1_SELECT_ZIVE_DATA_2026/AtsisiustiDuomenys_2026/KJ_-_2026-03-13_2225_to_2026-03-14_0636_8h_10min_test/KJ_-_2026-03-13_2225_to_2026-03-14_0636_8h_10min_test_records_summary.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Parameters" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Records'!$A$1:$AD$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Records'!$A$1:$AE$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD6"/>
+  <dimension ref="A1:AE6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -441,18 +441,19 @@
     <col width="10" customWidth="1" min="16" max="16"/>
     <col width="10" customWidth="1" min="17" max="17"/>
     <col width="10" customWidth="1" min="18" max="18"/>
-    <col width="12" customWidth="1" min="19" max="19"/>
-    <col width="10" customWidth="1" min="20" max="20"/>
+    <col width="10" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
     <col width="10" customWidth="1" min="21" max="21"/>
     <col width="10" customWidth="1" min="22" max="22"/>
     <col width="10" customWidth="1" min="23" max="23"/>
-    <col width="11" customWidth="1" min="24" max="24"/>
+    <col width="10" customWidth="1" min="24" max="24"/>
     <col width="11" customWidth="1" min="25" max="25"/>
-    <col width="13" customWidth="1" min="26" max="26"/>
-    <col width="10" customWidth="1" min="27" max="27"/>
-    <col width="26" customWidth="1" min="28" max="28"/>
+    <col width="11" customWidth="1" min="26" max="26"/>
+    <col width="13" customWidth="1" min="27" max="27"/>
+    <col width="10" customWidth="1" min="28" max="28"/>
     <col width="26" customWidth="1" min="29" max="29"/>
-    <col width="10" customWidth="1" min="30" max="30"/>
+    <col width="26" customWidth="1" min="30" max="30"/>
+    <col width="10" customWidth="1" min="31" max="31"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -523,85 +524,90 @@
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
+          <t>ectN</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
           <t>ectS</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>ectV</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>ectU</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>h_nz_cnt</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>h_nz_len</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>h_nz_frac%</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>out</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>rdr</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>noi</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>tp%</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>ml_nz_cnt</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>ml_nz_len</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>ml_nz_frac%</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>flags</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>recordingId</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>userId</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
@@ -646,17 +652,17 @@
         <v>3</v>
       </c>
       <c r="N2" t="n">
-        <v>0</v>
+        <v>692</v>
       </c>
       <c r="O2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" t="n">
         <v>2</v>
       </c>
-      <c r="P2" t="n">
+      <c r="Q2" t="n">
         <v>3</v>
       </c>
-      <c r="Q2" t="n">
-        <v>0</v>
-      </c>
       <c r="R2" t="n">
         <v>0</v>
       </c>
@@ -673,10 +679,10 @@
         <v>0</v>
       </c>
       <c r="W2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X2" t="n">
-        <v>0</v>
+        <v>2.7</v>
       </c>
       <c r="Y2" t="n">
         <v>0</v>
@@ -684,13 +690,16 @@
       <c r="Z2" t="n">
         <v>0</v>
       </c>
-      <c r="AA2" t="inlineStr"/>
-      <c r="AB2" t="inlineStr">
+      <c r="AA2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB2" t="inlineStr"/>
+      <c r="AC2" t="inlineStr">
         <is>
           <t>69b502078534dd1619e9670a</t>
         </is>
       </c>
-      <c r="AC2" t="inlineStr">
+      <c r="AD2" t="inlineStr">
         <is>
           <t>6072dcc694e6eac0851ab913</t>
         </is>
@@ -735,17 +744,17 @@
         <v>2</v>
       </c>
       <c r="N3" t="n">
+        <v>726</v>
+      </c>
+      <c r="O3" t="n">
         <v>1</v>
       </c>
-      <c r="O3" t="n">
-        <v>0</v>
-      </c>
       <c r="P3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" t="n">
         <v>2</v>
       </c>
-      <c r="Q3" t="n">
-        <v>0</v>
-      </c>
       <c r="R3" t="n">
         <v>0</v>
       </c>
@@ -759,13 +768,13 @@
         <v>0</v>
       </c>
       <c r="V3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W3" t="n">
         <v>8</v>
       </c>
-      <c r="W3" t="n">
-        <v>31.7</v>
-      </c>
       <c r="X3" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="Y3" t="n">
         <v>0</v>
@@ -773,13 +782,16 @@
       <c r="Z3" t="n">
         <v>0</v>
       </c>
-      <c r="AA3" t="inlineStr"/>
-      <c r="AB3" t="inlineStr">
+      <c r="AA3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB3" t="inlineStr"/>
+      <c r="AC3" t="inlineStr">
         <is>
           <t>69b5020f8534dd1619e96722</t>
         </is>
       </c>
-      <c r="AC3" t="inlineStr">
+      <c r="AD3" t="inlineStr">
         <is>
           <t>6072dcc694e6eac0851ab913</t>
         </is>
@@ -824,17 +836,17 @@
         <v>2</v>
       </c>
       <c r="N4" t="n">
+        <v>718</v>
+      </c>
+      <c r="O4" t="n">
         <v>1</v>
       </c>
-      <c r="O4" t="n">
-        <v>0</v>
-      </c>
       <c r="P4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" t="n">
         <v>2</v>
       </c>
-      <c r="Q4" t="n">
-        <v>0</v>
-      </c>
       <c r="R4" t="n">
         <v>0</v>
       </c>
@@ -848,27 +860,30 @@
         <v>0</v>
       </c>
       <c r="V4" t="n">
+        <v>0</v>
+      </c>
+      <c r="W4" t="n">
         <v>1</v>
       </c>
-      <c r="W4" t="n">
+      <c r="X4" t="n">
         <v>2.5</v>
       </c>
-      <c r="X4" t="n">
-        <v>0</v>
-      </c>
       <c r="Y4" t="n">
         <v>0</v>
       </c>
       <c r="Z4" t="n">
         <v>0</v>
       </c>
-      <c r="AA4" t="inlineStr"/>
-      <c r="AB4" t="inlineStr">
+      <c r="AA4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB4" t="inlineStr"/>
+      <c r="AC4" t="inlineStr">
         <is>
           <t>69b502108534dd1619e96724</t>
         </is>
       </c>
-      <c r="AC4" t="inlineStr">
+      <c r="AD4" t="inlineStr">
         <is>
           <t>6072dcc694e6eac0851ab913</t>
         </is>
@@ -913,17 +928,17 @@
         <v>3</v>
       </c>
       <c r="N5" t="n">
+        <v>475</v>
+      </c>
+      <c r="O5" t="n">
         <v>1</v>
       </c>
-      <c r="O5" t="n">
-        <v>0</v>
-      </c>
       <c r="P5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" t="n">
         <v>3</v>
       </c>
-      <c r="Q5" t="n">
-        <v>0</v>
-      </c>
       <c r="R5" t="n">
         <v>0</v>
       </c>
@@ -934,16 +949,16 @@
         <v>0</v>
       </c>
       <c r="U5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V5" t="n">
         <v>1</v>
       </c>
-      <c r="V5" t="n">
+      <c r="W5" t="n">
         <v>5</v>
       </c>
-      <c r="W5" t="n">
-        <v>62.7</v>
-      </c>
       <c r="X5" t="n">
-        <v>0</v>
+        <v>62.2</v>
       </c>
       <c r="Y5" t="n">
         <v>0</v>
@@ -951,13 +966,16 @@
       <c r="Z5" t="n">
         <v>0</v>
       </c>
-      <c r="AA5" t="inlineStr"/>
-      <c r="AB5" t="inlineStr">
+      <c r="AA5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB5" t="inlineStr"/>
+      <c r="AC5" t="inlineStr">
         <is>
           <t>69b5030f860fe9da479fc0e3</t>
         </is>
       </c>
-      <c r="AC5" t="inlineStr">
+      <c r="AD5" t="inlineStr">
         <is>
           <t>6072dcc694e6eac0851ab913</t>
         </is>
@@ -1002,17 +1020,17 @@
         <v>9</v>
       </c>
       <c r="N6" t="n">
-        <v>0</v>
+        <v>294</v>
       </c>
       <c r="O6" t="n">
         <v>0</v>
       </c>
       <c r="P6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" t="n">
         <v>10</v>
       </c>
-      <c r="Q6" t="n">
-        <v>0</v>
-      </c>
       <c r="R6" t="n">
         <v>0</v>
       </c>
@@ -1023,37 +1041,40 @@
         <v>0</v>
       </c>
       <c r="U6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V6" t="n">
         <v>4</v>
       </c>
-      <c r="V6" t="n">
-        <v>0</v>
-      </c>
       <c r="W6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X6" t="n">
         <v>39.5</v>
       </c>
-      <c r="X6" t="n">
-        <v>0</v>
-      </c>
       <c r="Y6" t="n">
         <v>0</v>
       </c>
       <c r="Z6" t="n">
         <v>0</v>
       </c>
-      <c r="AA6" t="inlineStr"/>
-      <c r="AB6" t="inlineStr">
+      <c r="AA6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB6" t="inlineStr"/>
+      <c r="AC6" t="inlineStr">
         <is>
           <t>69b50243860fe9da479fc0c9</t>
         </is>
       </c>
-      <c r="AC6" t="inlineStr">
+      <c r="AD6" t="inlineStr">
         <is>
           <t>6072dcc694e6eac0851ab913</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AD6"/>
+  <autoFilter ref="A1:AE6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1064,10 +1085,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -1105,6 +1126,31 @@
         <v>0.12</v>
       </c>
     </row>
+    <row r="4"/>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Ectopy model dir:</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>/home/kesju/DI/2025_ZIVEO/PROJECT_TRAIN_UNET/MODEL_VU_CNN</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Ectopy model:</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>best_model_final_2.keras</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add new scripts for updating records and modify existing data files
- Created `update_records_list_v6_GUNDAS.sh` for processing test data with denoising and ectopy configurations.
- Created `update_records_list_v6_POVILAS.sh` for processing data from Algirdo server with denoising and ectopy configurations.
- Updated binary files related to annotated records, including changes to `visi_zive_irasai_annot-Darb.xlsx` and removal of outdated files.
- Removed obsolete files: `visi_zive_irasai_annot_isplestas-Darb.xlsx`, `visi_zive_irasai_annot_isplestas-Darb_updated_1024_0_5_3_7_0_12.xlsx`, `zive_irasai_testui_isplestas.xlsx`, and `zive_irasai_testui_isplestas_updated_1024_0_5_3_7_0_12.xlsx`.
- Updated `zive_irasai_testui.xlsx` with new data.
</commit_message>
<xml_diff>
--- a/0_1_SELECT_ZIVE_DATA_2026/AtsisiustiDuomenys_2026/KJ_-_2026-03-13_2225_to_2026-03-14_0636_8h_10min_test/KJ_-_2026-03-13_2225_to_2026-03-14_0636_8h_10min_test_records_summary.xlsx
+++ b/0_1_SELECT_ZIVE_DATA_2026/AtsisiustiDuomenys_2026/KJ_-_2026-03-13_2225_to_2026-03-14_0636_8h_10min_test/KJ_-_2026-03-13_2225_to_2026-03-14_0636_8h_10min_test_records_summary.xlsx
@@ -437,9 +437,9 @@
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="10" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
+    <col hidden="1" width="10" customWidth="1" min="13" max="13"/>
+    <col hidden="1" width="10" customWidth="1" min="14" max="14"/>
+    <col hidden="1" width="10" customWidth="1" min="15" max="15"/>
     <col width="10" customWidth="1" min="16" max="16"/>
     <col width="10" customWidth="1" min="17" max="17"/>
     <col width="10" customWidth="1" min="18" max="18"/>
@@ -451,12 +451,12 @@
     <col width="10" customWidth="1" min="24" max="24"/>
     <col width="10" customWidth="1" min="25" max="25"/>
     <col width="10" customWidth="1" min="26" max="26"/>
-    <col width="11" customWidth="1" min="27" max="27"/>
-    <col width="11" customWidth="1" min="28" max="28"/>
-    <col width="26" customWidth="1" min="29" max="29"/>
-    <col width="26" customWidth="1" min="30" max="30"/>
-    <col width="13" customWidth="1" min="31" max="31"/>
-    <col width="10" customWidth="1" min="32" max="32"/>
+    <col hidden="1" width="11" customWidth="1" min="27" max="27"/>
+    <col hidden="1" width="11" customWidth="1" min="28" max="28"/>
+    <col hidden="1" width="13" customWidth="1" min="29" max="29"/>
+    <col width="10" customWidth="1" min="30" max="30"/>
+    <col width="26" customWidth="1" min="31" max="31"/>
+    <col width="26" customWidth="1" min="32" max="32"/>
     <col width="10" customWidth="1" min="33" max="33"/>
   </cols>
   <sheetData>
@@ -641,18 +641,12 @@
       <c r="C2" t="n">
         <v>128000</v>
       </c>
-      <c r="F2" t="n">
+      <c r="H2" t="n">
         <v>697</v>
       </c>
-      <c r="G2" t="n">
+      <c r="I2" t="n">
         <v>697</v>
       </c>
-      <c r="H2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0</v>
-      </c>
       <c r="J2" t="n">
         <v>0</v>
       </c>
@@ -663,26 +657,26 @@
         <v>0</v>
       </c>
       <c r="M2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" t="n">
         <v>3</v>
       </c>
-      <c r="N2" t="n">
+      <c r="P2" t="n">
         <v>692</v>
       </c>
-      <c r="O2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P2" t="n">
+      <c r="Q2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R2" t="n">
         <v>2</v>
       </c>
-      <c r="Q2" t="n">
+      <c r="S2" t="n">
         <v>3</v>
       </c>
-      <c r="R2" t="n">
-        <v>0</v>
-      </c>
-      <c r="S2" t="n">
-        <v>0</v>
-      </c>
       <c r="T2" t="n">
         <v>0</v>
       </c>
@@ -693,27 +687,33 @@
         <v>0</v>
       </c>
       <c r="W2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y2" t="n">
         <v>1</v>
       </c>
-      <c r="X2" t="n">
+      <c r="Z2" t="n">
         <v>2.7</v>
       </c>
-      <c r="Y2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z2" t="n">
-        <v>0</v>
-      </c>
       <c r="AA2" t="n">
         <v>0</v>
       </c>
-      <c r="AB2" t="inlineStr"/>
-      <c r="AC2" t="inlineStr">
+      <c r="AB2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD2" t="inlineStr"/>
+      <c r="AE2" t="inlineStr">
         <is>
           <t>69b502078534dd1619e9670a</t>
         </is>
       </c>
-      <c r="AD2" t="inlineStr">
+      <c r="AF2" t="inlineStr">
         <is>
           <t>6072dcc694e6eac0851ab913</t>
         </is>
@@ -733,48 +733,42 @@
       <c r="C3" t="n">
         <v>128000</v>
       </c>
-      <c r="F3" t="n">
+      <c r="H3" t="n">
         <v>729</v>
       </c>
-      <c r="G3" t="n">
+      <c r="I3" t="n">
         <v>729</v>
       </c>
-      <c r="H3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0</v>
-      </c>
       <c r="J3" t="n">
         <v>0</v>
       </c>
       <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" t="n">
         <v>1</v>
       </c>
-      <c r="L3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M3" t="n">
+      <c r="N3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" t="n">
         <v>2</v>
       </c>
-      <c r="N3" t="n">
+      <c r="P3" t="n">
         <v>726</v>
       </c>
-      <c r="O3" t="n">
+      <c r="Q3" t="n">
         <v>1</v>
       </c>
-      <c r="P3" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q3" t="n">
+      <c r="R3" t="n">
+        <v>0</v>
+      </c>
+      <c r="S3" t="n">
         <v>2</v>
       </c>
-      <c r="R3" t="n">
-        <v>0</v>
-      </c>
-      <c r="S3" t="n">
-        <v>0</v>
-      </c>
       <c r="T3" t="n">
         <v>0</v>
       </c>
@@ -785,27 +779,33 @@
         <v>0</v>
       </c>
       <c r="W3" t="n">
+        <v>0</v>
+      </c>
+      <c r="X3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y3" t="n">
         <v>8</v>
       </c>
-      <c r="X3" t="n">
+      <c r="Z3" t="n">
         <v>38</v>
       </c>
-      <c r="Y3" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z3" t="n">
-        <v>0</v>
-      </c>
       <c r="AA3" t="n">
         <v>0</v>
       </c>
-      <c r="AB3" t="inlineStr"/>
-      <c r="AC3" t="inlineStr">
+      <c r="AB3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD3" t="inlineStr"/>
+      <c r="AE3" t="inlineStr">
         <is>
           <t>69b5020f8534dd1619e96722</t>
         </is>
       </c>
-      <c r="AD3" t="inlineStr">
+      <c r="AF3" t="inlineStr">
         <is>
           <t>6072dcc694e6eac0851ab913</t>
         </is>
@@ -825,48 +825,42 @@
       <c r="C4" t="n">
         <v>128000</v>
       </c>
-      <c r="F4" t="n">
+      <c r="H4" t="n">
         <v>721</v>
       </c>
-      <c r="G4" t="n">
+      <c r="I4" t="n">
         <v>721</v>
       </c>
-      <c r="H4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" t="n">
-        <v>0</v>
-      </c>
       <c r="J4" t="n">
         <v>0</v>
       </c>
       <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" t="n">
         <v>1</v>
       </c>
-      <c r="L4" t="n">
-        <v>0</v>
-      </c>
-      <c r="M4" t="n">
+      <c r="N4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" t="n">
         <v>2</v>
       </c>
-      <c r="N4" t="n">
+      <c r="P4" t="n">
         <v>718</v>
       </c>
-      <c r="O4" t="n">
+      <c r="Q4" t="n">
         <v>1</v>
       </c>
-      <c r="P4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q4" t="n">
+      <c r="R4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S4" t="n">
         <v>2</v>
       </c>
-      <c r="R4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S4" t="n">
-        <v>0</v>
-      </c>
       <c r="T4" t="n">
         <v>0</v>
       </c>
@@ -877,27 +871,33 @@
         <v>0</v>
       </c>
       <c r="W4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y4" t="n">
         <v>1</v>
       </c>
-      <c r="X4" t="n">
+      <c r="Z4" t="n">
         <v>2.5</v>
       </c>
-      <c r="Y4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z4" t="n">
-        <v>0</v>
-      </c>
       <c r="AA4" t="n">
         <v>0</v>
       </c>
-      <c r="AB4" t="inlineStr"/>
-      <c r="AC4" t="inlineStr">
+      <c r="AB4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD4" t="inlineStr"/>
+      <c r="AE4" t="inlineStr">
         <is>
           <t>69b502108534dd1619e96724</t>
         </is>
       </c>
-      <c r="AD4" t="inlineStr">
+      <c r="AF4" t="inlineStr">
         <is>
           <t>6072dcc694e6eac0851ab913</t>
         </is>
@@ -917,48 +917,42 @@
       <c r="C5" t="n">
         <v>128000</v>
       </c>
-      <c r="F5" t="n">
+      <c r="H5" t="n">
         <v>471</v>
       </c>
-      <c r="G5" t="n">
+      <c r="I5" t="n">
         <v>471</v>
       </c>
-      <c r="H5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" t="n">
-        <v>0</v>
-      </c>
       <c r="J5" t="n">
         <v>0</v>
       </c>
       <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" t="n">
         <v>1</v>
       </c>
-      <c r="L5" t="n">
-        <v>0</v>
-      </c>
-      <c r="M5" t="n">
+      <c r="N5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" t="n">
         <v>3</v>
       </c>
-      <c r="N5" t="n">
+      <c r="P5" t="n">
         <v>475</v>
       </c>
-      <c r="O5" t="n">
+      <c r="Q5" t="n">
         <v>1</v>
       </c>
-      <c r="P5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q5" t="n">
+      <c r="R5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S5" t="n">
         <v>3</v>
       </c>
-      <c r="R5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S5" t="n">
-        <v>0</v>
-      </c>
       <c r="T5" t="n">
         <v>0</v>
       </c>
@@ -966,30 +960,36 @@
         <v>0</v>
       </c>
       <c r="V5" t="n">
+        <v>0</v>
+      </c>
+      <c r="W5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X5" t="n">
         <v>1</v>
       </c>
-      <c r="W5" t="n">
+      <c r="Y5" t="n">
         <v>5</v>
       </c>
-      <c r="X5" t="n">
+      <c r="Z5" t="n">
         <v>62.2</v>
       </c>
-      <c r="Y5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z5" t="n">
-        <v>0</v>
-      </c>
       <c r="AA5" t="n">
         <v>0</v>
       </c>
-      <c r="AB5" t="inlineStr"/>
-      <c r="AC5" t="inlineStr">
+      <c r="AB5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD5" t="inlineStr"/>
+      <c r="AE5" t="inlineStr">
         <is>
           <t>69b5030f860fe9da479fc0e3</t>
         </is>
       </c>
-      <c r="AD5" t="inlineStr">
+      <c r="AF5" t="inlineStr">
         <is>
           <t>6072dcc694e6eac0851ab913</t>
         </is>
@@ -1009,18 +1009,12 @@
       <c r="C6" t="n">
         <v>128000</v>
       </c>
-      <c r="F6" t="n">
+      <c r="H6" t="n">
         <v>274</v>
       </c>
-      <c r="G6" t="n">
+      <c r="I6" t="n">
         <v>274</v>
       </c>
-      <c r="H6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" t="n">
-        <v>0</v>
-      </c>
       <c r="J6" t="n">
         <v>0</v>
       </c>
@@ -1031,26 +1025,26 @@
         <v>0</v>
       </c>
       <c r="M6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" t="n">
         <v>9</v>
       </c>
-      <c r="N6" t="n">
+      <c r="P6" t="n">
         <v>294</v>
       </c>
-      <c r="O6" t="n">
-        <v>0</v>
-      </c>
-      <c r="P6" t="n">
-        <v>0</v>
-      </c>
       <c r="Q6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S6" t="n">
         <v>10</v>
       </c>
-      <c r="R6" t="n">
-        <v>0</v>
-      </c>
-      <c r="S6" t="n">
-        <v>0</v>
-      </c>
       <c r="T6" t="n">
         <v>0</v>
       </c>
@@ -1058,30 +1052,36 @@
         <v>0</v>
       </c>
       <c r="V6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X6" t="n">
         <v>4</v>
       </c>
-      <c r="W6" t="n">
-        <v>0</v>
-      </c>
-      <c r="X6" t="n">
+      <c r="Y6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z6" t="n">
         <v>39.5</v>
       </c>
-      <c r="Y6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z6" t="n">
-        <v>0</v>
-      </c>
       <c r="AA6" t="n">
         <v>0</v>
       </c>
-      <c r="AB6" t="inlineStr"/>
-      <c r="AC6" t="inlineStr">
+      <c r="AB6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD6" t="inlineStr"/>
+      <c r="AE6" t="inlineStr">
         <is>
           <t>69b50243860fe9da479fc0c9</t>
         </is>
       </c>
-      <c r="AD6" t="inlineStr">
+      <c r="AF6" t="inlineStr">
         <is>
           <t>6072dcc694e6eac0851ab913</t>
         </is>

</xml_diff>